<commit_message>
feat(#58): optional DataType column in config sheets for explicit type annotation
Add dataTypeColIdx header.findIndex lookup in mapSheet(). For non-asset
rows, DataType value overrides inferred cell type when present and
recognised (string/int/double/bool/DateOnly/DateTime/TimeOnly).
Falls back to getCellWithType() inference when column is absent,
empty, or value is unrecognised — no breaking change.

Config_Reference.xlsx Settings sheet gains DataType column; SampleRate
row demonstrates int cell forced to double via explicit DataType.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/Config_Reference.xlsx
+++ b/test/fixtures/Config_Reference.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -523,6 +523,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>DataType</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -574,58 +579,78 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IsEnabled</t>
-        </is>
-      </c>
-      <c r="B5" t="b">
-        <v>1</v>
+          <t>SampleRate</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bool — Master feature toggle.</t>
+          <t>double forced via DataType (cell is int).</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>double</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CutoffDate</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46022</v>
+          <t>IsEnabled</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DateOnly — Last valid processing date.</t>
+          <t>bool — Master feature toggle.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ScheduledAt</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>45823.39583333334</v>
+          <t>CutoffDate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46022</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DateTime — Next scheduled run.</t>
+          <t>DateOnly — Last valid processing date.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>ScheduledAt</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>45823.39583333334</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DateTime — Next scheduled run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>DailyRunTime</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B9" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>TimeOnly — Daily start time.</t>
         </is>

</xml_diff>

<commit_message>
feat: _ prefix convention, per-file meta overrides, generator version header, and ToXxx() default guards (#90, #57)
- Hard migrate directive prefix from . to _ for TOML parity (breaking):
  sheet filter, _TargetType row, _Meta sheet, generate_fixtures.py, all docs
- Per-file settings overrides via _Meta sheet (xlsx) or [_meta] table (TOML):
  readMetaSheet, readTomlMeta; resetConfigToStored + applyMetaOverrides on upload;
  setConfigValue extracted as shared helper; [_Meta] case-insensitive match
- _TargetType parity for TOML: _ -prefixed keys in parseTomlNode are directives
- <auto-generated> header in every generated .cs file (VERSION file, version.js, #57)
- ToXxx() guards string defaults: IsNullOrEmpty fallback for non-empty string defaults
- defaultValue threaded through all parsers (xlsx, TOML, JSON)
- All 16 golden fixtures updated

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/Config_Reference.xlsx
+++ b/test/fixtures/Config_Reference.xlsx
@@ -7,14 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name=".Meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_Meta" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Constants" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Environments" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Features" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Assets" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Connections" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name=".Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="_Notes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1362,24 +1362,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>.Meta</t>
+          <t>_Meta</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hidden — excluded from code generation (dot prefix).</t>
+          <t>Hidden — excluded from code generation (underscore prefix).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>.Notes</t>
+          <t>_Notes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hidden — excluded from code generation (dot prefix).</t>
+          <t>Hidden — excluded from code generation (underscore prefix).</t>
         </is>
       </c>
     </row>

</xml_diff>